<commit_message>
chnaged 150Ohms to 390
</commit_message>
<xml_diff>
--- a/8Bit Computer ver2.0/excel/BOM.xlsx
+++ b/8Bit Computer ver2.0/excel/BOM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\home\Desktop\Computer_HTL\8Bit Computer ver2.0\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DIP\8Bit_Computer\8Bit Computer ver2.0\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B876FACF-DE5A-4BD4-8B25-768C788652C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{037D1D16-AB4F-4799-833D-3299CBBF5C8B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F82DDFF1-7D1A-40D7-BAFF-AC1E2824F50D}"/>
   </bookViews>
@@ -17,21 +17,12 @@
     <sheet name="Tabelle1" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="ExterneDaten_1" localSheetId="0" hidden="1">'Computer'!$B:$D</definedName>
+    <definedName name="ExterneDaten_1" localSheetId="0" hidden="1">Computer!$B:$D</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -46,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="199">
   <si>
     <t>Reference</t>
   </si>
@@ -591,9 +582,6 @@
     <t>R72,R73,R74,R75,R76,R77,R78,R79,R80,R81,R82,R83,R84,R85,R86,R87,R88,R89,R90,R91,R92,R93,R94,R95,R96,R97,R98,R99,R100,R101,R102,R103,R104,R105,R106,R107,R108,R109,R110,R111</t>
   </si>
   <si>
-    <t>150</t>
-  </si>
-  <si>
     <t>S1,S2,S14</t>
   </si>
   <si>
@@ -640,6 +628,12 @@
   </si>
   <si>
     <t>Crystal:Crystal_SMD_HC49-SD_HandSoldering</t>
+  </si>
+  <si>
+    <t>x40</t>
+  </si>
+  <si>
+    <t>72+40</t>
   </si>
 </sst>
 </file>
@@ -1938,8 +1932,8 @@
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53">
-        <v>72</v>
+      <c r="A53" t="s">
+        <v>198</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>169</v>
@@ -2040,11 +2034,11 @@
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59">
-        <v>40</v>
-      </c>
-      <c r="B59" s="1" t="s">
-        <v>181</v>
+      <c r="A59" t="s">
+        <v>197</v>
+      </c>
+      <c r="B59" s="1">
+        <v>150</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>159</v>
@@ -2061,16 +2055,16 @@
         <v>3</v>
       </c>
       <c r="B60" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="C60" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="C60" s="1" t="s">
+      <c r="D60" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="D60" s="1" t="s">
-        <v>185</v>
-      </c>
       <c r="E60" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
@@ -2078,16 +2072,16 @@
         <v>11</v>
       </c>
       <c r="B61" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C61" s="1" t="s">
         <v>187</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>188</v>
       </c>
       <c r="D61" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
@@ -2098,13 +2092,13 @@
         <v>8</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D62" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
@@ -2112,16 +2106,16 @@
         <v>1</v>
       </c>
       <c r="B63" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C63" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="C63" s="1" t="s">
+      <c r="D63" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="D63" s="1" t="s">
-        <v>194</v>
-      </c>
       <c r="E63" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
@@ -2129,16 +2123,16 @@
         <v>1</v>
       </c>
       <c r="B64" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="C64" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="C64" s="1" t="s">
-        <v>197</v>
-      </c>
       <c r="D64" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>

</xml_diff>